<commit_message>
add further soft constraint
</commit_message>
<xml_diff>
--- a/java/shiftsolver/testSmall.xlsx
+++ b/java/shiftsolver/testSmall.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\milan\code\ShiftSolver\java\shiftsolver\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D667BCD3-4C28-4F9E-92DA-5C5328EC4FE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9513D5BE-0A06-4C62-B72E-0E9D672C61E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-75" yWindow="-16320" windowWidth="29040" windowHeight="15990" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Einstellungen" sheetId="5" r:id="rId1"/>
@@ -994,7 +994,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1238,44 +1238,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="43" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="23" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="2" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="9" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1292,6 +1255,42 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="9" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1668,7 +1667,7 @@
     <col min="1" max="1" width="20.77734375" customWidth="1"/>
     <col min="2" max="2" width="11.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="70.88671875" customWidth="1"/>
-    <col min="4" max="4" width="18" style="95" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -1677,10 +1676,10 @@
       </c>
       <c r="B1" s="83"/>
       <c r="C1" s="83"/>
-      <c r="D1" s="100"/>
+      <c r="D1" s="87"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="105" t="s">
+      <c r="A2" s="92" t="s">
         <v>25</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1689,7 +1688,7 @@
       <c r="C2" s="41" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="96"/>
+      <c r="D2" s="85"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -1731,7 +1730,7 @@
       <c r="B6" s="3">
         <v>10</v>
       </c>
-      <c r="C6" s="99" t="s">
+      <c r="C6" s="86" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1742,17 +1741,17 @@
       <c r="B7" s="3">
         <v>4.5</v>
       </c>
-      <c r="C7" s="99" t="s">
+      <c r="C7" s="86" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="102" t="s">
+      <c r="A8" s="89" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="101"/>
-      <c r="C8" s="103"/>
-      <c r="D8" s="100"/>
+      <c r="B8" s="88"/>
+      <c r="C8" s="90"/>
+      <c r="D8" s="87"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
@@ -1780,10 +1779,10 @@
       </c>
       <c r="B11" s="84"/>
       <c r="C11" s="84"/>
-      <c r="D11" s="100"/>
+      <c r="D11" s="87"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="104" t="s">
+      <c r="A12" s="91" t="s">
         <v>26</v>
       </c>
       <c r="B12" t="s">
@@ -1792,12 +1791,12 @@
       <c r="C12" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="95" t="s">
+      <c r="D12" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="104" t="s">
+      <c r="A13" s="91" t="s">
         <v>28</v>
       </c>
       <c r="B13" t="s">
@@ -1805,7 +1804,7 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="104" t="s">
+      <c r="A14" s="91" t="s">
         <v>29</v>
       </c>
       <c r="B14" t="s">
@@ -1813,7 +1812,7 @@
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="104" t="s">
+      <c r="A15" s="91" t="s">
         <v>30</v>
       </c>
       <c r="B15" t="s">
@@ -1821,7 +1820,7 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="104" t="s">
+      <c r="A16" s="91" t="s">
         <v>31</v>
       </c>
       <c r="B16" t="s">
@@ -1880,7 +1879,7 @@
       <c r="H1" s="32"/>
     </row>
     <row r="2" spans="1:285" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="85">
+      <c r="A2" s="97">
         <v>45597</v>
       </c>
       <c r="B2" s="55" t="s">
@@ -1888,35 +1887,31 @@
       </c>
       <c r="C2" s="45">
         <f t="shared" ref="C2:C35" si="0">COUNTIF(D2:G2,"&gt;1")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" s="44">
         <v>7</v>
       </c>
       <c r="E2" s="43"/>
-      <c r="F2" s="44">
-        <v>7</v>
-      </c>
+      <c r="F2" s="44"/>
       <c r="G2" s="44"/>
       <c r="H2" s="34"/>
       <c r="I2" s="26"/>
     </row>
     <row r="3" spans="1:285" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="86"/>
+      <c r="A3" s="102"/>
       <c r="B3" s="54" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="46">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" s="15">
         <v>10</v>
       </c>
       <c r="E3" s="10"/>
-      <c r="F3" s="15">
-        <v>10</v>
-      </c>
+      <c r="F3" s="15"/>
       <c r="G3" s="15"/>
       <c r="H3" s="34"/>
       <c r="I3" s="26"/>
@@ -2198,7 +2193,7 @@
       <c r="JY3"/>
     </row>
     <row r="4" spans="1:285" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="90">
+      <c r="A4" s="103">
         <f>A2+1</f>
         <v>45598</v>
       </c>
@@ -2212,35 +2207,31 @@
       <c r="D4" s="8">
         <v>7</v>
       </c>
-      <c r="E4" s="11"/>
+      <c r="E4" s="11">
+        <v>7</v>
+      </c>
       <c r="F4" s="8">
         <v>7</v>
       </c>
-      <c r="G4" s="8">
-        <v>7</v>
-      </c>
+      <c r="G4" s="8"/>
       <c r="H4" s="32"/>
       <c r="I4" s="26"/>
     </row>
     <row r="5" spans="1:285" s="2" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="91"/>
+      <c r="A5" s="104"/>
       <c r="B5" s="17" t="s">
         <v>7</v>
       </c>
       <c r="C5" s="46">
         <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="D5" s="49"/>
-      <c r="E5" s="12">
+        <v>1</v>
+      </c>
+      <c r="D5" s="49">
         <v>10</v>
       </c>
-      <c r="F5" s="14">
-        <v>10</v>
-      </c>
-      <c r="G5" s="14">
-        <v>10</v>
-      </c>
+      <c r="E5" s="12"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
       <c r="H5" s="32"/>
       <c r="I5" s="26"/>
       <c r="J5"/>
@@ -2521,7 +2512,7 @@
       <c r="JY5"/>
     </row>
     <row r="6" spans="1:285" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="90">
+      <c r="A6" s="103">
         <f>A4+1</f>
         <v>45599</v>
       </c>
@@ -2544,7 +2535,7 @@
       <c r="I6" s="26"/>
     </row>
     <row r="7" spans="1:285" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="91"/>
+      <c r="A7" s="104"/>
       <c r="B7" s="17" t="s">
         <v>3</v>
       </c>
@@ -2842,7 +2833,7 @@
       <c r="JY7"/>
     </row>
     <row r="8" spans="1:285" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="88">
+      <c r="A8" s="98">
         <f>A6+1</f>
         <v>45600</v>
       </c>
@@ -2851,12 +2842,10 @@
       </c>
       <c r="C8" s="46">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D8" s="50"/>
-      <c r="E8" s="9">
-        <v>3.5</v>
-      </c>
+      <c r="E8" s="9"/>
       <c r="F8" s="9">
         <v>3.5</v>
       </c>
@@ -2867,24 +2856,20 @@
       <c r="I8" s="26"/>
     </row>
     <row r="9" spans="1:285" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="89"/>
+      <c r="A9" s="99"/>
       <c r="B9" s="17" t="s">
         <v>3</v>
       </c>
       <c r="C9" s="46">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D9" s="49"/>
       <c r="E9" s="13">
         <v>7.5</v>
       </c>
-      <c r="F9" s="13">
-        <v>7.5</v>
-      </c>
-      <c r="G9" s="13">
-        <v>7.5</v>
-      </c>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
       <c r="H9" s="32"/>
       <c r="I9" s="26"/>
       <c r="J9"/>
@@ -3165,7 +3150,7 @@
       <c r="JY9"/>
     </row>
     <row r="10" spans="1:285" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="87">
+      <c r="A10" s="93">
         <f>A8+1</f>
         <v>45601</v>
       </c>
@@ -3174,32 +3159,28 @@
       </c>
       <c r="C10" s="46">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" s="48"/>
       <c r="E10" s="11">
         <v>3.5</v>
       </c>
-      <c r="F10" s="11">
-        <v>3.5</v>
-      </c>
+      <c r="F10" s="11"/>
       <c r="G10" s="11"/>
       <c r="H10" s="36"/>
       <c r="I10" s="26"/>
     </row>
     <row r="11" spans="1:285" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="87"/>
+      <c r="A11" s="93"/>
       <c r="B11" s="17" t="s">
         <v>3</v>
       </c>
       <c r="C11" s="46">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" s="49"/>
-      <c r="E11" s="13">
-        <v>7.5</v>
-      </c>
+      <c r="E11" s="13"/>
       <c r="F11" s="13">
         <v>7.5</v>
       </c>
@@ -3484,7 +3465,7 @@
       <c r="JY11"/>
     </row>
     <row r="12" spans="1:285" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="87">
+      <c r="A12" s="93">
         <f>A10+1</f>
         <v>45602</v>
       </c>
@@ -3505,7 +3486,7 @@
       <c r="I12" s="26"/>
     </row>
     <row r="13" spans="1:285" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="87"/>
+      <c r="A13" s="93"/>
       <c r="B13" s="17" t="s">
         <v>3</v>
       </c>
@@ -3799,7 +3780,7 @@
       <c r="JY13"/>
     </row>
     <row r="14" spans="1:285" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="87">
+      <c r="A14" s="93">
         <f>A12+1</f>
         <v>45603</v>
       </c>
@@ -3822,7 +3803,7 @@
       <c r="I14" s="26"/>
     </row>
     <row r="15" spans="1:285" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="87"/>
+      <c r="A15" s="93"/>
       <c r="B15" s="20" t="s">
         <v>3</v>
       </c>
@@ -4118,7 +4099,7 @@
       <c r="JY15"/>
     </row>
     <row r="16" spans="1:285" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="87">
+      <c r="A16" s="93">
         <f>A14+1</f>
         <v>45604</v>
       </c>
@@ -4141,7 +4122,7 @@
       <c r="I16" s="27"/>
     </row>
     <row r="17" spans="1:291" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="87"/>
+      <c r="A17" s="93"/>
       <c r="B17" s="20" t="s">
         <v>7</v>
       </c>
@@ -4163,7 +4144,7 @@
       <c r="I17" s="28"/>
     </row>
     <row r="18" spans="1:291" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="92">
+      <c r="A18" s="96">
         <f>A16+1</f>
         <v>45605</v>
       </c>
@@ -4186,7 +4167,7 @@
       <c r="I18" s="26"/>
     </row>
     <row r="19" spans="1:291" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="92"/>
+      <c r="A19" s="96"/>
       <c r="B19" s="21" t="s">
         <v>7</v>
       </c>
@@ -4206,7 +4187,7 @@
       <c r="I19" s="26"/>
     </row>
     <row r="20" spans="1:291" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="92">
+      <c r="A20" s="96">
         <f>A18+1</f>
         <v>45606</v>
       </c>
@@ -4229,7 +4210,7 @@
       <c r="I20" s="26"/>
     </row>
     <row r="21" spans="1:291" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="92"/>
+      <c r="A21" s="96"/>
       <c r="B21" s="20" t="s">
         <v>3</v>
       </c>
@@ -4251,7 +4232,7 @@
       <c r="I21" s="26"/>
     </row>
     <row r="22" spans="1:291" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="87">
+      <c r="A22" s="93">
         <f>A20+1</f>
         <v>45607</v>
       </c>
@@ -4276,7 +4257,7 @@
       <c r="I22" s="26"/>
     </row>
     <row r="23" spans="1:291" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="87"/>
+      <c r="A23" s="93"/>
       <c r="B23" s="20" t="s">
         <v>3</v>
       </c>
@@ -4298,7 +4279,7 @@
       <c r="I23" s="26"/>
     </row>
     <row r="24" spans="1:291" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="87">
+      <c r="A24" s="93">
         <f>A22+1</f>
         <v>45608</v>
       </c>
@@ -4323,7 +4304,7 @@
       <c r="I24" s="26"/>
     </row>
     <row r="25" spans="1:291" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="87"/>
+      <c r="A25" s="93"/>
       <c r="B25" s="25" t="s">
         <v>3</v>
       </c>
@@ -4345,7 +4326,7 @@
       <c r="I25" s="26"/>
     </row>
     <row r="26" spans="1:291" s="4" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="87">
+      <c r="A26" s="93">
         <f>A24+1</f>
         <v>45609</v>
       </c>
@@ -4652,7 +4633,7 @@
       <c r="KE26" s="29"/>
     </row>
     <row r="27" spans="1:291" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="87"/>
+      <c r="A27" s="93"/>
       <c r="B27" s="17" t="s">
         <v>3</v>
       </c>
@@ -4673,7 +4654,7 @@
       <c r="H27" s="40"/>
     </row>
     <row r="28" spans="1:291" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="88">
+      <c r="A28" s="98">
         <f>A26+1</f>
         <v>45610</v>
       </c>
@@ -4697,7 +4678,7 @@
       <c r="H28" s="33"/>
     </row>
     <row r="29" spans="1:291" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="89"/>
+      <c r="A29" s="99"/>
       <c r="B29" s="20" t="s">
         <v>3</v>
       </c>
@@ -4718,7 +4699,7 @@
       <c r="H29" s="33"/>
     </row>
     <row r="30" spans="1:291" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="93">
+      <c r="A30" s="100">
         <f>A28+1</f>
         <v>45611</v>
       </c>
@@ -4742,7 +4723,7 @@
       <c r="H30" s="33"/>
     </row>
     <row r="31" spans="1:291" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="94"/>
+      <c r="A31" s="101"/>
       <c r="B31" s="20" t="s">
         <v>7</v>
       </c>
@@ -4763,7 +4744,7 @@
       <c r="H31" s="33"/>
     </row>
     <row r="32" spans="1:291" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="92">
+      <c r="A32" s="96">
         <f>A30+1</f>
         <v>45612</v>
       </c>
@@ -4787,7 +4768,7 @@
       <c r="H32" s="33"/>
     </row>
     <row r="33" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="92"/>
+      <c r="A33" s="96"/>
       <c r="B33" s="17" t="s">
         <v>7</v>
       </c>
@@ -4808,7 +4789,7 @@
       <c r="H33" s="33"/>
     </row>
     <row r="34" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="92">
+      <c r="A34" s="96">
         <f>A32+1</f>
         <v>45613</v>
       </c>
@@ -4832,7 +4813,7 @@
       <c r="H34" s="33"/>
     </row>
     <row r="35" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="85"/>
+      <c r="A35" s="97"/>
       <c r="B35" s="79" t="s">
         <v>3</v>
       </c>
@@ -4861,10 +4842,10 @@
       <c r="H36" s="33"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A37" s="97" t="s">
+      <c r="A37" s="94" t="s">
         <v>27</v>
       </c>
-      <c r="B37" s="98"/>
+      <c r="B37" s="95"/>
       <c r="C37" s="64" t="s">
         <v>11</v>
       </c>
@@ -4883,8 +4864,8 @@
       <c r="H37" s="32"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A38" s="97"/>
-      <c r="B38" s="98"/>
+      <c r="A38" s="94"/>
+      <c r="B38" s="95"/>
       <c r="C38" s="65" t="s">
         <v>12</v>
       </c>
@@ -4903,26 +4884,26 @@
       <c r="H38" s="32"/>
     </row>
     <row r="39" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="97"/>
-      <c r="B39" s="98"/>
+      <c r="A39" s="94"/>
+      <c r="B39" s="95"/>
       <c r="C39" s="62" t="s">
         <v>13</v>
       </c>
       <c r="D39" s="76">
         <f>SUM(D2:D35)</f>
-        <v>155.5</v>
+        <v>165.5</v>
       </c>
       <c r="E39" s="77">
         <f>SUM(E2:E35)</f>
-        <v>158</v>
+        <v>144</v>
       </c>
       <c r="F39" s="77">
         <f>SUM(F2:F35)</f>
-        <v>120</v>
+        <v>82</v>
       </c>
       <c r="G39" s="78">
         <f>SUM(G2:G35)</f>
-        <v>153.5</v>
+        <v>129</v>
       </c>
       <c r="H39" s="32"/>
     </row>
@@ -4958,6 +4939,13 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="A12:A13"/>
     <mergeCell ref="A16:A17"/>
     <mergeCell ref="A37:B39"/>
     <mergeCell ref="A34:A35"/>
@@ -4969,13 +4957,6 @@
     <mergeCell ref="A24:A25"/>
     <mergeCell ref="A30:A31"/>
     <mergeCell ref="A32:A33"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="A12:A13"/>
   </mergeCells>
   <conditionalFormatting sqref="C2:C35">
     <cfRule type="colorScale" priority="2">

</xml_diff>